<commit_message>
more attempts in training, added some datasets
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -400,6 +400,12 @@
     </xf>
     <xf numFmtId="16" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -407,12 +413,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -744,18 +744,18 @@
     </row>
     <row r="2" spans="1:14" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:14" ht="109.2" x14ac:dyDescent="0.3">
@@ -787,7 +787,7 @@
       <c r="L3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="15" t="s">
         <v>19</v>
       </c>
     </row>
@@ -961,7 +961,7 @@
         <f t="shared" si="0"/>
         <v>0.32471428571428573</v>
       </c>
-      <c r="N8" s="18">
+      <c r="N8" s="15">
         <v>0.33200000000000002</v>
       </c>
     </row>
@@ -978,7 +978,7 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="2"/>
-      <c r="N9" s="17"/>
+      <c r="N9" s="14"/>
     </row>
     <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
@@ -995,7 +995,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="2"/>
-      <c r="N10" s="17"/>
+      <c r="N10" s="14"/>
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
@@ -1081,18 +1081,18 @@
     </row>
     <row r="15" spans="1:14" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="16"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="18"/>
       <c r="L15" s="2"/>
     </row>
     <row r="16" spans="1:14" ht="109.2" x14ac:dyDescent="0.3">
@@ -1368,7 +1368,6 @@
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1381,7 +1380,6 @@
     <row r="27" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -1432,21 +1430,21 @@
     </row>
     <row r="2" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="s">
@@ -1475,7 +1473,7 @@
       <c r="L3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="15" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1577,7 +1575,7 @@
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N8" s="18"/>
+      <c r="N8" s="15"/>
     </row>
     <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -1592,7 +1590,7 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="2"/>
-      <c r="N9" s="17"/>
+      <c r="N9" s="14"/>
     </row>
     <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
@@ -1609,7 +1607,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="2"/>
-      <c r="N10" s="17"/>
+      <c r="N10" s="14"/>
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
@@ -1695,18 +1693,18 @@
     </row>
     <row r="15" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="16"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="18"/>
       <c r="L15" s="2"/>
     </row>
     <row r="16" spans="1:14" ht="93.6" x14ac:dyDescent="0.3">

</xml_diff>